<commit_message>
Troubleshoot MCCTrip On Off problem
</commit_message>
<xml_diff>
--- a/Reference/Merge Table UI.xlsx
+++ b/Reference/Merge Table UI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A33E8F0-619E-490D-9DBE-9460DA7FCFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC14C926-6CAD-4138-9215-983B2ED69D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{31D85F91-40ED-4F68-9A5B-7EC9EBBDCEBE}"/>
   </bookViews>
@@ -414,8 +414,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4165,22 +4165,22 @@
       <c r="E4" t="s">
         <v>78</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="G4" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -4200,22 +4200,22 @@
       <c r="E5" t="s">
         <v>78</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="G5" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -6925,23 +6925,23 @@
     <col min="1" max="6" width="17.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
All quota model empty
</commit_message>
<xml_diff>
--- a/Reference/Merge Table UI.xlsx
+++ b/Reference/Merge Table UI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC14C926-6CAD-4138-9215-983B2ED69D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1A040F-14FC-457C-86D5-05FE49ADCBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{31D85F91-40ED-4F68-9A5B-7EC9EBBDCEBE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="6" xr2:uid="{31D85F91-40ED-4F68-9A5B-7EC9EBBDCEBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -4515,22 +4515,22 @@
       <c r="E14" t="s">
         <v>87</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G14" t="s">
-        <v>76</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="G14" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J14" t="s">
-        <v>76</v>
-      </c>
-      <c r="K14" t="s">
+      <c r="J14" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K14" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4550,22 +4550,22 @@
       <c r="E15" t="s">
         <v>87</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G15" t="s">
-        <v>76</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="G15" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4585,22 +4585,22 @@
       <c r="E16" t="s">
         <v>88</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G16" t="s">
-        <v>76</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="G16" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J16" t="s">
-        <v>76</v>
-      </c>
-      <c r="K16" t="s">
+      <c r="J16" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K16" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4620,22 +4620,22 @@
       <c r="E17" t="s">
         <v>88</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G17" t="s">
-        <v>76</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="G17" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4725,22 +4725,22 @@
       <c r="E20" t="s">
         <v>89</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G20" t="s">
-        <v>76</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="G20" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K20" t="s">
+      <c r="J20" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4760,22 +4760,22 @@
       <c r="E21" t="s">
         <v>89</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G21" t="s">
-        <v>76</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="G21" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K21" t="s">
+      <c r="K21" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4795,22 +4795,22 @@
       <c r="E22" t="s">
         <v>90</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G22" t="s">
-        <v>76</v>
-      </c>
-      <c r="H22" t="s">
+      <c r="G22" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J22" t="s">
-        <v>76</v>
-      </c>
-      <c r="K22" t="s">
+      <c r="J22" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K22" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4830,22 +4830,22 @@
       <c r="E23" t="s">
         <v>90</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G23" t="s">
-        <v>76</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="G23" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H23" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K23" t="s">
+      <c r="K23" s="5" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove 2 models from Groq Llama due to free-tier access restrictions
</commit_message>
<xml_diff>
--- a/Reference/Merge Table UI.xlsx
+++ b/Reference/Merge Table UI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1A040F-14FC-457C-86D5-05FE49ADCBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E43D1D8-278F-484D-8A30-C809F0FDACAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="6" xr2:uid="{31D85F91-40ED-4F68-9A5B-7EC9EBBDCEBE}"/>
   </bookViews>
@@ -6922,7 +6922,9 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="6" width="17.08984375" customWidth="1"/>
+    <col min="1" max="2" width="17.08984375" customWidth="1"/>
+    <col min="3" max="3" width="37.7265625" customWidth="1"/>
+    <col min="4" max="6" width="17.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>